<commit_message>
Napi adatok, HTML és hidegtárolási Excel-exportok frissítése
</commit_message>
<xml_diff>
--- a/data/garazstarolas_export.xlsx
+++ b/data/garazstarolas_export.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Aptos Narrow"/>
       <charset val="238"/>
@@ -29,8 +29,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="004DA3FF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +51,11 @@
         <fgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B9BD5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -60,10 +69,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -461,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:G105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="2"/>
@@ -470,6 +481,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,7 +512,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Tárolás helye</t>
+          <t>Terv tárolás</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Tény tárolás</t>
         </is>
       </c>
     </row>
@@ -530,7 +547,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -562,7 +584,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -594,7 +621,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -626,7 +658,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -658,7 +695,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -690,7 +732,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F7" s="1" t="inlineStr">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -722,7 +769,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F8" s="1" t="inlineStr">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -754,7 +806,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -786,7 +843,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F10" s="1" t="inlineStr">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -818,7 +880,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -850,7 +917,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -882,7 +954,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -914,7 +991,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr">
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -946,7 +1028,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr">
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -978,7 +1065,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr">
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1010,7 +1102,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F17" s="1" t="inlineStr">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1042,7 +1139,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F18" s="1" t="inlineStr">
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1074,7 +1176,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F19" s="1" t="inlineStr">
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G19" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1106,7 +1213,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F20" s="1" t="inlineStr">
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1138,7 +1250,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F21" s="1" t="inlineStr">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1170,7 +1287,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1202,7 +1324,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F23" s="1" t="inlineStr">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1234,7 +1361,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1266,7 +1398,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr">
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G25" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1298,7 +1435,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G26" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1330,7 +1472,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr">
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1362,7 +1509,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G28" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1394,7 +1546,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr">
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G29" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -1426,7 +1583,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr">
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G30" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1458,7 +1620,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F31" s="1" t="inlineStr">
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G31" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1490,7 +1657,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F32" s="1" t="inlineStr">
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1522,7 +1694,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F33" s="1" t="inlineStr">
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G33" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1554,7 +1731,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F34" s="1" t="inlineStr">
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G34" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -1586,7 +1768,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F35" s="1" t="inlineStr">
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1618,7 +1805,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F36" s="1" t="inlineStr">
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1645,14 +1837,19 @@
           <t>AOIM035</t>
         </is>
       </c>
-      <c r="E37" s="1" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="F37" s="1" t="inlineStr">
-        <is>
-          <t>ArrivaBus Andor telephely</t>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1879,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F38" s="1" t="inlineStr">
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G38" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1714,7 +1916,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F39" s="1" t="inlineStr">
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1746,7 +1953,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F40" s="1" t="inlineStr">
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G40" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -1778,7 +1990,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F41" s="1" t="inlineStr">
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1810,7 +2027,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F42" s="1" t="inlineStr">
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1842,7 +2064,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F43" s="1" t="inlineStr">
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G43" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -1874,7 +2101,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F44" s="1" t="inlineStr">
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G44" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1906,7 +2138,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F45" s="1" t="inlineStr">
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -1938,7 +2175,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F46" s="1" t="inlineStr">
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -1970,7 +2212,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F47" s="1" t="inlineStr">
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G47" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2002,7 +2249,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F48" s="1" t="inlineStr">
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2034,7 +2286,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F49" s="1" t="inlineStr">
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2066,7 +2323,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F50" s="1" t="inlineStr">
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G50" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2098,7 +2360,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F51" s="1" t="inlineStr">
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2130,7 +2397,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F52" s="1" t="inlineStr">
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2162,7 +2434,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F53" s="1" t="inlineStr">
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2194,7 +2471,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F54" s="1" t="inlineStr">
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2226,7 +2508,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F55" s="1" t="inlineStr">
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G55" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2258,7 +2545,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F56" s="1" t="inlineStr">
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2290,7 +2582,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F57" s="1" t="inlineStr">
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2322,7 +2619,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F58" s="1" t="inlineStr">
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G58" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2354,7 +2656,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F59" s="1" t="inlineStr">
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G59" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2386,7 +2693,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F60" s="1" t="inlineStr">
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G60" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2418,7 +2730,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F61" s="1" t="inlineStr">
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G61" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2450,7 +2767,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F62" s="1" t="inlineStr">
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -2482,7 +2804,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F63" s="1" t="inlineStr">
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2514,7 +2841,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F64" s="1" t="inlineStr">
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G64" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2546,7 +2878,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F65" s="1" t="inlineStr">
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G65" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -2578,7 +2915,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F66" s="1" t="inlineStr">
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G66" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2610,7 +2952,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F67" s="1" t="inlineStr">
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G67" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2642,7 +2989,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F68" s="1" t="inlineStr">
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G68" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2674,7 +3026,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F69" s="1" t="inlineStr">
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G69" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2706,7 +3063,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F70" s="1" t="inlineStr">
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2738,7 +3100,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F71" s="1" t="inlineStr">
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G71" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2770,7 +3137,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F72" s="1" t="inlineStr">
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G72" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2802,7 +3174,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F73" s="1" t="inlineStr">
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G73" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2834,7 +3211,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F74" s="1" t="inlineStr">
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G74" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2866,7 +3248,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F75" s="1" t="inlineStr">
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G75" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2898,7 +3285,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F76" s="1" t="inlineStr">
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G76" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -2930,7 +3322,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F77" s="1" t="inlineStr">
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G77" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -2962,7 +3359,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F78" s="1" t="inlineStr">
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G78" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -2994,7 +3396,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F79" s="1" t="inlineStr">
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G79" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -3026,7 +3433,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F80" s="1" t="inlineStr">
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G80" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3058,7 +3470,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F81" s="1" t="inlineStr">
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G81" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -3090,7 +3507,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F82" s="1" t="inlineStr">
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G82" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -3122,7 +3544,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F83" s="1" t="inlineStr">
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G83" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3154,7 +3581,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F84" s="1" t="inlineStr">
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G84" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3186,7 +3618,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F85" s="1" t="inlineStr">
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G85" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3218,7 +3655,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F86" s="1" t="inlineStr">
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G86" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -3250,7 +3692,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F87" s="1" t="inlineStr">
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G87" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -3282,7 +3729,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F88" s="1" t="inlineStr">
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G88" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3314,7 +3766,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F89" s="1" t="inlineStr">
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G89" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3346,7 +3803,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F90" s="1" t="inlineStr">
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G90" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3378,7 +3840,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F91" s="1" t="inlineStr">
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G91" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3410,7 +3877,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F92" s="1" t="inlineStr">
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G92" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3442,7 +3914,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F93" s="1" t="inlineStr">
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G93" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3474,7 +3951,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F94" s="1" t="inlineStr">
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G94" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -3506,7 +3988,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F95" s="1" t="inlineStr">
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G95" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3538,7 +4025,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F96" s="1" t="inlineStr">
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G96" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -3570,7 +4062,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F97" s="1" t="inlineStr">
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G97" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -3602,7 +4099,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F98" s="1" t="inlineStr">
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G98" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3634,7 +4136,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F99" s="1" t="inlineStr">
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="G99" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Szállító telephely</t>
         </is>
@@ -3666,7 +4173,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F100" s="1" t="inlineStr">
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G100" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3698,7 +4210,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F101" s="1" t="inlineStr">
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G101" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Andor telephely</t>
         </is>
@@ -3730,7 +4247,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F102" s="1" t="inlineStr">
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G102" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3757,14 +4279,19 @@
           <t>AOGL316</t>
         </is>
       </c>
-      <c r="E103" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="F103" s="2" t="inlineStr">
-        <is>
-          <t>47.40818, 19.016005</t>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>---</t>
         </is>
       </c>
     </row>
@@ -3794,7 +4321,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F104" s="1" t="inlineStr">
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G104" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>
@@ -3826,7 +4358,12 @@
           <t>I</t>
         </is>
       </c>
-      <c r="F105" s="1" t="inlineStr">
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="G105" s="1" t="inlineStr">
         <is>
           <t>ArrivaBus Bogáncs telephely</t>
         </is>

</xml_diff>

<commit_message>
Napi adatok, HTML, archívum és hidegtárolási Excel-exportok frissítése
</commit_message>
<xml_diff>
--- a/data/garazstarolas_export.xlsx
+++ b/data/garazstarolas_export.xlsx
@@ -34,7 +34,7 @@
       <color rgb="004DA3FF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -51,6 +51,14 @@
         <fgColor rgb="005B9BD5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid"/>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -64,11 +72,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -466,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G105"/>
+  <dimension ref="A1:G209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="2"/>
@@ -4363,6 +4373,3850 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>AOIM034</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F106" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G106" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1012</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>PDN607</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F107" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G107" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>AOIM037</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F108" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G108" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>AAMH666</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F109" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G109" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>AOIM027</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>n.a</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1840</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>SGY814</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F111" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G111" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1012</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>PDN640</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F112" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G112" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>AAMH664</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F113" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G113" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>0310</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>AAMH673</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F114" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G114" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>AOIM036</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F115" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G115" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1820</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>SGY815</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F116" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G116" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>0205</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>AAMH665</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F117" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G117" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1240</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>AAHY844</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F118" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G118" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>0350</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>SGY808</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F119" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G119" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>AAHY845</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F120" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G120" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>AOIM029</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>AOIM049</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F122" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G122" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>0660</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>AOIM056</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F123" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G123" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1225</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>AAMH679</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F124" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G124" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>AOIA477</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F125" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G125" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1240</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>AAHY820</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F126" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G126" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>0205</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>AAMH642</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F127" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G127" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>AOIB822</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F128" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G128" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1140</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>AOGL314</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F129" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G129" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1012</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>PDN601</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G130" s="4" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>AAMH619</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F131" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G131" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1225</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>AAMH626</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F132" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G132" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>0350</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>SGY810</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F133" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G133" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>AAMH610</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G134" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>0960</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>AAHY848</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F135" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G135" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>2120</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>AOIA474</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F136" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G136" s="4" t="inlineStr">
+        <is>
+          <t>47.478207, 18.840927</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>0205</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>AAMH676</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F137" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G137" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>0660</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>AOGF651</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F138" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G138" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>1390</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>AONW963</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F139" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G139" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>AOIA475</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F140" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G140" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>AOIM035</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F141" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G141" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>AOIM045</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F142" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G142" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>0205</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>AAMH651</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F143" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G143" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1480</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>AOJM871</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F144" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G144" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>0960</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>AAHY879</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F145" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G145" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1012</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>PDN603</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F146" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G146" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>AOIM046</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F147" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G147" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>AOLH516</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F148" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G148" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>1225</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>AAMH680</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F149" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G149" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1820</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>PDN627</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F150" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G150" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>AAMH678</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F151" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G151" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>AOCT655</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F152" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G152" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>0310</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>AAMH603</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F153" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G153" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>AOGL311</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F154" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G154" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>0205</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>AOCT651</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F155" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G155" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr"/>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F156" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>n.a</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>0250</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>AAHY866</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F157" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G157" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>AAMH622</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F158" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G158" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>AOIM028</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F159" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G159" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>1390</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>AOIM044</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F160" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G160" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2200</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>AAHY867</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F161" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G161" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>AOCT656</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F162" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G162" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>1012</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>PDN602</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F163" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G163" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>AOIM033</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F164" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G164" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>1380</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>PDN630</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G165" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>1510</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>AOGF670</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F166" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G166" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>AOCT666</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F167" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G167" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>AAMH663</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F168" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G168" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>1840</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>SGY823</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F169" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G169" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>1012</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>PDN604</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F170" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G170" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2120</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>AOIA471</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F171" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G171" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>AOCT673</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F172" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G172" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>AOIM053</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F173" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G173" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>1470</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>AAHY801</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F174" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G174" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1530</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>PDN632</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F175" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G175" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>1390</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>AOIM026</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F176" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G176" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>AOIM043</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F177" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G177" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>1040</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>AAHY834</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F178" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G178" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>AOGL305</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F179" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G179" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>2235</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>AOJM867</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F180" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G180" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2120</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>AOIA470</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F181" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G181" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>1335</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>AOCT669</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F182" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G182" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>1590</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>AOJM886</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F183" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G183" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>1225</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>AAHY854</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F184" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G184" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>1390</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>AOIB826</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F185" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G185" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>1530</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>PDN631</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F186" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G186" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>1240</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>AAHY826</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F187" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G187" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>1040</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>AAHY837</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F188" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G188" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>AAMH674</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F189" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G189" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>1590</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>AOJM885</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F190" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G190" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>2120</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>AOIB804</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F191" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G191" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>AAMH634</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F192" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G192" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>AAHY859</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F193" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G193" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>AOLH515</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F194" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G194" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>AOCT675</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F195" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G195" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>1040</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>AAHY836</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F196" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G196" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>1470</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>AAHY849</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F197" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G197" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>0530</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>PDN610</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G198" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>0205</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>AAMH617</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F199" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G199" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>1530</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>VTA641</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F200" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G200" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2120</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>PDN638</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F201" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G201" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>0205</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>AAMH616</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F202" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G202" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>0660</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>AOGF652</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+      <c r="F203" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G203" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Szállító telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>AADR720</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G204" s="3" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>1390</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>AONW951</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F205" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G205" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>1240</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>AAHY880</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F206" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G206" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>AOGL316</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+      <c r="F207" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G207" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Andor telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>1100</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>AOCT671</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F208" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G208" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>0085</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>AOCT657</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+      <c r="F209" s="1" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="G209" s="1" t="inlineStr">
+        <is>
+          <t>ArrivaBus Bogáncs telephely</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>